<commit_message>
Implement sitemap processing and Excel handling services
- Add sitemap_service.py for downloading and parsing sitemaps.
- Introduce excel_service.py for creating and managing Excel workbooks.
- Create markdown_service.py for fetching and extracting markdown content from webpages.
- Implement path_service.py for generating safe file paths and slugs from URLs.
- Add semantic_router_service.py for routing markdown based on user needs using a language model.
- Define PipelineState in state.py to manage input values and file paths.
</commit_message>
<xml_diff>
--- a/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
+++ b/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D151"/>
+  <dimension ref="A1:G153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,21 @@
           <t>markdown_status</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>similarity_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>semantic_status</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>semantic_reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -459,6 +474,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E2" t="n">
+        <v>34</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Focuses on software-defined vehicles and trust, not electric vehicle manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -481,6 +509,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E3" t="n">
+        <v>72</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>About EV production performance and delivery growth, relevant to electric vehicle manufacturing.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -503,6 +544,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E4" t="n">
+        <v>88</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>About EV market expansion, dealers, tariffs, and possible manufacturing investment in North American automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -525,6 +579,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E5" t="n">
+        <v>82</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and Toyota’s domestic supply chain labor needs.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -547,6 +614,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E6" t="n">
+        <v>74</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and OEM supply chains through LiDAR production, supplier relationships, and vehicle program adoption.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -569,6 +649,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E7" t="n">
+        <v>91</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>About a new automotive manufacturing plant and supplier investment for GM’s vehicle platform.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -591,6 +684,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E8" t="n">
+        <v>19</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>About in-car media software, not electric vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -613,6 +719,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E9" t="n">
+        <v>57</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>About bus service center construction, not electric vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -635,6 +754,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E10" t="n">
+        <v>93</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Article is about EV battery development, automaker partnerships, and the automotive supply chain.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -657,6 +789,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and supply-chain recycling/circularity.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -679,6 +824,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E12" t="n">
+        <v>86</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>About EV manufacturing plans, production targets, and factory construction.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -701,6 +859,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E13" t="n">
+        <v>29</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Board appointment news, not about EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -723,6 +894,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E14" t="n">
+        <v>52</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Mentions mostly electric vehicles and transport contracts, which is somewhat related to automotive supply and EV manufacturing.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -745,6 +929,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E15" t="n">
+        <v>95</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Discusses GM manufacturing investment, EV retooling, and automotive production supply-chain implications.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -767,6 +964,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E16" t="n">
+        <v>62</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>About Audi corporate transformation, not EV manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -789,6 +999,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E17" t="n">
+        <v>72</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Relevant to automotive technology and OEM vehicle platforms, though not specifically manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -811,6 +1034,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E18" t="n">
+        <v>89</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>About automotive supplier innovations for EVs and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -833,6 +1069,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E19" t="n">
+        <v>34</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>It is an OEM model launch article, not about EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -855,6 +1104,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E20" t="n">
+        <v>78</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Discusses EV manufacturing strategy and dependence on Honda’s automotive platform and supply chain.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -877,6 +1139,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E21" t="n">
+        <v>93</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Directly about EV battery recycling and automotive manufacturing supply-chain compliance.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -899,6 +1174,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E22" t="n">
+        <v>68</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Relevant to EV charging infrastructure and parts/service support in the automotive ecosystem.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -921,6 +1209,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E23" t="n">
+        <v>18</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>It is about vehicle safety awards, not EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -943,6 +1244,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E24" t="n">
+        <v>68</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>About bus manufacturing and vehicle deliveries in Brazil, which is related to automotive manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -965,6 +1279,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E25" t="n">
+        <v>42</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Relevant to commercial vehicles, but not directly about EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -987,6 +1314,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E26" t="n">
+        <v>22</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>About eBike services and digital mobility, not electric vehicle manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1009,6 +1349,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E27" t="n">
+        <v>62</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Includes an electric vehicle reveal and a commercial van tied to an automaker, which is somewhat relevant to EV manufacturing and automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1031,6 +1384,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E28" t="n">
+        <v>18</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>About Mazda safety awards, not electric vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1053,6 +1419,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E29" t="n">
+        <v>87</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Relevant to electric vehicle manufacturing and automotive supply chains through electric trucks, fleet electrification, and charging infrastructure.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1075,6 +1454,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E30" t="n">
+        <v>88</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>About an electric vehicle launch for fleets, directly related to EV manufacturing and automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1097,6 +1489,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E31" t="n">
+        <v>12</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>It is a vehicle performance announcement, not about EV manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1119,6 +1524,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E32" t="n">
+        <v>18</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>A new SUV teaser is not about EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1141,6 +1559,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E33" t="n">
+        <v>74</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Relevant EV manufacturing news with production details and supply-chain-adjacent battery/platform information.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1163,6 +1594,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E34" t="n">
+        <v>17</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>About EV charging infrastructure, not manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1185,6 +1629,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E35" t="n">
+        <v>12</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>About rideshare toll software, not EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1207,6 +1664,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E36" t="n">
+        <v>68</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Relevant to vehicle manufacturing and electrified commercial-vehicle products, though not directly about automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1229,6 +1699,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E37" t="n">
+        <v>74</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and supplier relations, with EV strategy and supply chain impacts.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1251,6 +1734,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E38" t="n">
+        <v>72</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>About automotive market strategy and EV competition, with some relevance to manufacturing and supply-chain shifts.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1273,6 +1769,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E39" t="n">
+        <v>88</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Covers Hyundai’s vehicle production expansion and regional supply chain investment, which is relevant to automotive manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1295,6 +1804,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E40" t="n">
+        <v>18</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Focuses on ADAS safety claims for Mazda, not EV manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1317,6 +1839,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E41" t="n">
+        <v>38</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>About OEM safety technology, not electric vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1339,6 +1874,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E42" t="n">
+        <v>95</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Directly about automotive supply chains and manufacturing.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1361,6 +1909,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E43" t="n">
+        <v>87</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>About BMW manufacturing, recycling, battery supply, and vehicle materials in the automotive supply chain.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1383,6 +1944,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E44" t="n">
+        <v>70</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and factory operations, though focused more on robotics and labour relations than supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1405,6 +1979,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E45" t="n">
+        <v>73</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Relevant to automotive industry operations and OEM brand/channel strategy, though not specifically about manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1427,6 +2014,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E46" t="n">
+        <v>74</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Relevant to EV manufacturing via Hyundai electric vehicle and automotive product design wins.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1449,6 +2049,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E47" t="n">
+        <v>74</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and supply chain disruptions affecting GM production.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1471,6 +2084,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E48" t="n">
+        <v>39</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Focuses on robotaxi services and autonomy, not electric vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1493,6 +2119,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E49" t="n">
+        <v>41</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>About an automaker’s new hybrid model, not specifically manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1515,6 +2154,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E50" t="n">
+        <v>28</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Article is mainly about Corvette performance models, only loosely related to automotive manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1537,6 +2189,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E51" t="n">
+        <v>92</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Directly covers EV-related vehicle manufacturing and automotive supply-chain localization in North America.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1559,6 +2224,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E52" t="n">
+        <v>86</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>About EV production at Audi FAW NEV and production/logistics, which fits automotive manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1581,6 +2259,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E53" t="n">
+        <v>18</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>About autonomous vehicle safety research, not electric vehicle manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1603,6 +2294,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E54" t="n">
+        <v>31</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>About robotaxi/autonomous ride-hailing, not EV manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1625,6 +2329,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E55" t="n">
+        <v>74</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Relevant to automotive technology and supplier testing for vehicle networking.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1647,6 +2364,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E56" t="n">
+        <v>82</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>About EV sales, OEM product plans, and automotive market changes.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1669,6 +2399,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E57" t="n">
+        <v>72</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>About battery supply for electric vehicles and a Chinese light EV maker, which fits EV manufacturing and supply chain relevance.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1691,6 +2434,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E58" t="n">
+        <v>72</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>About EV charging network operations, which is relevant to automotive supply chain and EV industry articles.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1713,6 +2469,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E59" t="n">
+        <v>72</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Relevant to electric vehicles and OEM automotive news, though not directly about manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1735,6 +2504,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E60" t="n">
+        <v>88</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>About an electric vehicle model and its production for delivery fleets, relevant to EV manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1757,6 +2539,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E61" t="n">
+        <v>18</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>About ride-hailing and chauffeur services, with only a brief EV mention and no automotive manufacturing or supply-chain focus.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1779,6 +2574,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E62" t="n">
+        <v>58</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>About EV manufacturing strategy and OEM supply chain/JV dynamics.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1801,6 +2609,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E63" t="n">
+        <v>92</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>About automotive manufacturing and recycled material supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1823,6 +2644,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E64" t="n">
+        <v>82</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Relevant to electric vehicle manufacturing and OEM software platform development in the automotive supply chain.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1845,6 +2679,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E65" t="n">
+        <v>18</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>About AI customer feedback analysis, not electric vehicle manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1867,6 +2714,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E66" t="n">
+        <v>96</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>About EV production at a manufacturing plant and automotive output.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1889,6 +2749,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E67" t="n">
+        <v>18</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>About Mazda ADAS safety research, not electric vehicle manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1911,6 +2784,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E68" t="n">
+        <v>12</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>About a new Infiniti SUV launch, not EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1933,6 +2819,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E69" t="n">
+        <v>92</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Discusses automakers, manufacturing costs, and supply chain disruptions affecting vehicle production.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1955,6 +2854,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E70" t="n">
+        <v>96</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Directly about electric vehicle production and an automotive manufacturing supply chain partnership.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1977,6 +2889,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E71" t="n">
+        <v>72</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Relevant to automakers and vehicle software supply chains, though not directly about EV manufacturing.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1999,6 +2924,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E72" t="n">
+        <v>78</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Discusses Tesla EV manufacturing and OEM performance, relevant to automotive supply chain context.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2021,6 +2959,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E73" t="n">
+        <v>91</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>About auto manufacturing, supplier disruption, and vehicle production supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2043,6 +2994,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E74" t="n">
+        <v>94</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>About automotive manufacturing investment and production in the EV/e-mobility supply chain context.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2065,6 +3029,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E75" t="n">
+        <v>78</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>About automotive R&amp;D and vehicle platform development for Geely brands, relevant to manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2087,6 +3064,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E76" t="n">
+        <v>78</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Discusses Volkswagen manufacturing parts and broader automotive supply chain implications.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2109,6 +3099,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E77" t="n">
+        <v>86</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Relevant to electric vehicle manufacturing and an automotive supply-chain partnership between Rivian and Volkswagen.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2131,6 +3134,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E78" t="n">
+        <v>68</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and supplier strategy, though it focuses on bus exports and market expansion rather than EV-specific supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2153,6 +3169,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E79" t="n">
+        <v>84</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Relevant to automotive supply chains and vehicle manufacturing, with heavy vehicle fleet renewal and domestic producer support.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2175,6 +3204,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E80" t="n">
+        <v>31</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>About EV charging infrastructure and standards, not vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2197,6 +3239,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E81" t="n">
+        <v>97</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>About EV battery production and vehicle manufacturing within an automotive supply chain.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2219,6 +3274,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E82" t="n">
+        <v>87</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>About OEM distribution and spare-parts logistics in Europe, relevant to automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2241,6 +3309,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E83" t="n">
+        <v>72</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Relevant to automotive supply chains and vehicle manufacturing software/sensor integration.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2263,6 +3344,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E84" t="n">
+        <v>72</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Relevant to automotive supply chains and OEM/supplier support, though not directly about EV manufacturing.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2285,6 +3379,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E85" t="n">
+        <v>88</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>About an automaker’s manufacturing operations and data systems, relevant to automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2307,6 +3414,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E86" t="n">
+        <v>84</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Relevant to electric vehicle manufacturing and OEM supply-chain activity.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2329,6 +3449,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E87" t="n">
+        <v>84</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>About truck OEM leadership tied to Fuso-Hino integration, relevant to automotive supply chain and manufacturing.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2351,6 +3484,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E88" t="n">
+        <v>94</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Directly about an automotive OEM’s global shipping and supply chain for vehicle exports.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2373,6 +3519,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E89" t="n">
+        <v>78</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Relevant to electric vehicle manufacturing and commercial vehicle supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2395,6 +3554,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E90" t="n">
+        <v>95</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Directly about EV battery materials and the automotive EV supply chain.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2417,6 +3589,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E91" t="n">
+        <v>12</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>About ride-hailing and premium travel, not EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2439,6 +3624,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E92" t="n">
+        <v>82</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>About an EV automaker and subsidy impacts on automotive market supply conditions.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2461,6 +3659,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E93" t="n">
+        <v>89</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Volkswagen production forecasts and OEM outlook are directly relevant to automotive manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2483,6 +3694,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E94" t="n">
+        <v>78</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Relevant to EV manufacturing and automotive market/supply-chain dynamics, especially subsidies affecting OEM competition.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2505,6 +3729,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E95" t="n">
+        <v>84</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>It discusses electric vehicle development and manufacturing of an EV in India.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2517,10 +3754,20 @@
           <t>2026-03-31T07:29:14+00:00</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>failed</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>source_missing</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Markdown path is missing.</t>
         </is>
       </c>
     </row>
@@ -2545,6 +3792,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E97" t="n">
+        <v>18</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>About luxury car demand and shipment disruptions, not EV manufacturing or broader automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2567,6 +3827,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E98" t="n">
+        <v>93</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>About an EV maker’s overseas manufacturing expansion and global automotive supply chain footprint.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2589,6 +3862,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E99" t="n">
+        <v>38</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>About an SUV launch and EV tech, not manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2611,6 +3897,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E100" t="n">
+        <v>72</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Relevant to automotive supply chains and vehicle manufacturing technology.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2633,6 +3932,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E101" t="n">
+        <v>82</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Relevant to automotive supply chains and European vehicle distribution.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2655,6 +3967,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E102" t="n">
+        <v>22</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Focuses on Musk/Tesla legal disputes, not EV manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2677,6 +4002,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E103" t="n">
+        <v>88</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Tesla manufacturing leadership and EV production ramp are directly relevant to electric vehicle manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2699,6 +4037,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E104" t="n">
+        <v>88</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>About automakers collaborating on fuel cell technology and transport supply chain development.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2721,6 +4072,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E105" t="n">
+        <v>94</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Discusses EV manufacturing, production shift to US, and automotive supply chain implications.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2743,6 +4107,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E106" t="n">
+        <v>92</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>About automotive manufacturing technology for vehicle paint shops and energy-efficient production.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2765,6 +4142,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E107" t="n">
+        <v>92</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>About electric vehicle manufacturing and a logistics/automotive fleet supply order.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2787,6 +4177,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E108" t="n">
+        <v>94</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>The article directly concerns EV manufacturing and automotive production shifts within a supply chain context.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2809,6 +4212,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E109" t="n">
+        <v>12</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>It is about a design award for a Fiat model, not EV manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2831,6 +4247,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E110" t="n">
+        <v>14</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>About autonomous ride-hailing in Tokyo, not electric vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2853,6 +4282,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E111" t="n">
+        <v>72</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and supply-chain collaboration in commercial vehicle fuel cell production.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2875,6 +4317,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E112" t="n">
+        <v>18</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>About vehicle sales forecasting, not EV manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2897,6 +4352,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E113" t="n">
+        <v>94</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>About Denso’s automotive manufacturing, electrification, and supply chain-related industrial production.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2919,6 +4387,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E114" t="n">
+        <v>88</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>About BEV manufacturing and a battery production facility in an automaker’s supply chain.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2941,6 +4422,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E115" t="n">
+        <v>57</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and EV transition, though focused on heavy-duty vehicle CO2 rules rather than supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2963,6 +4457,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E116" t="n">
+        <v>72</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Relevant EV OEM news; less about manufacturing or supply chains directly.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2985,6 +4492,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E117" t="n">
+        <v>84</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>It discusses Toyota production and manufacturing, which is relevant to automotive supply chains and vehicle manufacturing.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3007,6 +4527,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E118" t="n">
+        <v>67</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and EV mobility, though not directly about supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3029,6 +4562,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E119" t="n">
+        <v>82</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Article covers EV production at Mercedes-Benz’s Alabama plant and broader automotive manufacturing operations.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3051,6 +4597,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E120" t="n">
+        <v>72</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Relevant to electric vehicle manufacturing and OEM vehicle platform news, with some commercial vehicle context.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3073,6 +4632,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E121" t="n">
+        <v>12</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>About autonomous robotaxi service, not electric vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3095,6 +4667,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E122" t="n">
+        <v>42</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>About commercial vehicle software platforms, not electric vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3117,6 +4702,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E123" t="n">
+        <v>41</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>It is about in-car software and entertainment, not vehicle manufacturing or supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3139,6 +4737,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E124" t="n">
+        <v>22</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>It’s about transportation infrastructure and LiDAR, not electric vehicle manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3161,6 +4772,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E125" t="n">
+        <v>18</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>About autonomous robotaxis and software outage, not EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3183,6 +4807,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E126" t="n">
+        <v>41</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>About digital key software and vehicle access, only loosely related to EV manufacturing and supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3205,6 +4842,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E127" t="n">
+        <v>84</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Relevant to automotive supply chains and commercial vehicle manufacturing.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3227,6 +4877,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E128" t="n">
+        <v>12</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>About autonomous ride services, not electric vehicle manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3249,6 +4912,19 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E129" t="n">
+        <v>89</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>About commercial vehicle OEM integration, shared procurement and production, and zero-emission technologies.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3271,143 +4947,234 @@
           <t>success</t>
         </is>
       </c>
+      <c r="E130" t="n">
+        <v>12</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>About in-vehicle navigation software, not EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/news/volvo-trucks-begins-road-testing-hydrogen-combustion-trucks/</t>
+          <t>https://www.automotiveworld.com/news/macron-courts-asian-battery-makers-on-east-asia-tour/</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-04-01T07:48:03+00:00</t>
+          <t>2026-04-01T08:22:32+00:00</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/volvo-trucks-begins-road-testing-hydrogen-combustion-trucks.md</t>
+          <t>scraped_markdown/automotiveworld/macron-courts-asian-battery-makers-on-east-asia-tour.md</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>95</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Article is directly about EV battery manufacturing and supply chain localization.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/news/audi-introduces-torque-vectoring-world-first-in-rs-5/</t>
+          <t>https://www.automotiveworld.com/news/volvo-trucks-begins-road-testing-hydrogen-combustion-trucks/</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-04-01T07:50:42+00:00</t>
+          <t>2026-04-01T08:53:15+00:00</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/audi-introduces-torque-vectoring-world-first-in-rs-5.md</t>
+          <t>scraped_markdown/automotiveworld/volvo-trucks-begins-road-testing-hydrogen-combustion-trucks.md</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>72</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Relevant to automotive manufacturing and vehicle powertrain technology, though not directly about supply chains.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/media-specifications/</t>
+          <t>https://www.automotiveworld.com/news/audi-introduces-torque-vectoring-world-first-in-rs-5/</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-03-25T17:23:22+00:00</t>
+          <t>2026-04-01T08:53:25+00:00</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/media-specifications.md</t>
+          <t>scraped_markdown/automotiveworld/audi-introduces-torque-vectoring-world-first-in-rs-5.md</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>18</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>About a specific Audi performance vehicle feature, not manufacturing or supply chains.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/editorial-calendar/</t>
+          <t>https://www.automotiveworld.com/news/ntsb-faults-fords-adas-tech-in-two-fatal-highway-crashes/</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-03-31T15:21:54+00:00</t>
+          <t>2026-04-01T09:01:45+00:00</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/editorial-calendar.md</t>
+          <t>scraped_markdown/automotiveworld/ntsb-faults-fords-adas-tech-in-two-fatal-highway-crashes.md</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>22</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>About ADAS safety, not electric vehicle manufacturing or automotive supply chains.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/mp-files/</t>
+          <t>https://www.automotiveworld.com/media-specifications/</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-03-31T09:35:12+00:00</t>
+          <t>2026-03-25T17:23:22+00:00</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/mp-files.md</t>
+          <t>scraped_markdown/automotiveworld/media-specifications.md</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>3</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>This page is about advertising media specifications, not articles on EV manufacturing or automotive supply chains.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/mp-files/volkswagen-group-profile-and-production-forecast-to-2030.xlsx/</t>
+          <t>https://www.automotiveworld.com/editorial-calendar/</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-03-30T10:19:06+00:00</t>
+          <t>2026-03-31T15:21:54+00:00</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/volkswagen-group-profile-and-production-forecast-to-2030.xlsx.md</t>
+          <t>scraped_markdown/automotiveworld/editorial-calendar.md</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>79</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Contains automotive industry items on vehicle production, manufacturers, and plant databases relevant to supply chains.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/mp-files/toyota-profile-and-production-forecast-to-2030.xlsx/</t>
+          <t>https://www.automotiveworld.com/mp-files/</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3417,320 +5184,585 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/toyota-profile-and-production-forecast-to-2030.xlsx.md</t>
+          <t>scraped_markdown/automotiveworld/mp-files.md</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>72</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Contains automotive-industry content and events on software-defined vehicles and OEM development, relevant to automotive supply chains and EV manufacturing context.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/analysis/</t>
+          <t>https://www.automotiveworld.com/mp-files/volkswagen-group-profile-and-production-forecast-to-2030.xlsx/</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-03-31T18:12:09+00:00</t>
+          <t>2026-03-30T10:19:06+00:00</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/analysis.md</t>
+          <t>scraped_markdown/automotiveworld/volkswagen-group-profile-and-production-forecast-to-2030.xlsx.md</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>8</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>This is a login/subscription page, not an article about EV manufacturing or supply chains.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/articles/</t>
+          <t>https://www.automotiveworld.com/mp-files/toyota-profile-and-production-forecast-to-2030.xlsx/</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-04-01T06:46:39+00:00</t>
+          <t>2026-03-31T09:35:12+00:00</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/articles.md</t>
+          <t>scraped_markdown/automotiveworld/toyota-profile-and-production-forecast-to-2030.xlsx.md</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>5</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Login page only; no article content about EV manufacturing or supply chains.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/autonomous-driving/</t>
+          <t>https://www.automotiveworld.com/analysis/</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-04-01T06:57:59+00:00</t>
+          <t>2026-03-31T18:12:09+00:00</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/autonomous-driving.md</t>
+          <t>scraped_markdown/automotiveworld/analysis.md</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>72</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>The page is Automotive World analysis content about OEMs and suppliers, which is broadly relevant to automotive supply chains.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/commercial-vehicle/</t>
+          <t>https://www.automotiveworld.com/articles/</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-04-01T07:48:03+00:00</t>
+          <t>2026-04-01T06:46:39+00:00</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/commercial-vehicle.md</t>
+          <t>scraped_markdown/automotiveworld/articles.md</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>78</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>The page is about automotive trends including electrification, which is relevant to EV manufacturing and supply chains.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/data/</t>
+          <t>https://www.automotiveworld.com/topics/autonomous-driving/</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-03-31T15:32:04+00:00</t>
+          <t>2026-04-01T09:01:45+00:00</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/data.md</t>
+          <t>scraped_markdown/automotiveworld/autonomous-driving.md</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>18</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Page is about autonomous driving, not EV manufacturing or automotive supply chains.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/e-mobility/</t>
+          <t>https://www.automotiveworld.com/topics/commercial-vehicle/</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-04-01T07:50:42+00:00</t>
+          <t>2026-04-01T08:53:15+00:00</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/e-mobility.md</t>
+          <t>scraped_markdown/automotiveworld/commercial-vehicle.md</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>52</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Commercial vehicles and electrification are somewhat relevant to EV manufacturing and supply chains.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/manufacturing/</t>
+          <t>https://www.automotiveworld.com/data/</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-03-31T18:57:48+00:00</t>
+          <t>2026-03-31T15:32:04+00:00</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/manufacturing.md</t>
+          <t>scraped_markdown/automotiveworld/data.md</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>42</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>This page is a data listings page, not articles about EV manufacturing or supply chains.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/markets/</t>
+          <t>https://www.automotiveworld.com/topics/e-mobility/</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-04-01T06:57:59+00:00</t>
+          <t>2026-04-01T08:53:25+00:00</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/markets.md</t>
+          <t>scraped_markdown/automotiveworld/e-mobility.md</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>79</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>The page is about E-Mobility and mentions EVs, battery technology, and market dynamics relevant to automotive manufacturing and supply chains.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/news/</t>
+          <t>https://www.automotiveworld.com/topics/manufacturing/</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-04-01T07:50:42+00:00</t>
+          <t>2026-04-01T08:22:32+00:00</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/news.md</t>
+          <t>scraped_markdown/automotiveworld/manufacturing.md</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>87</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Manufacturing topic page covers automotive production and supply chains, which matches the need.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/data/oem-outlooks/</t>
+          <t>https://www.automotiveworld.com/topics/markets/</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-03-30T13:13:27+00:00</t>
+          <t>2026-04-01T09:01:45+00:00</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/oem-outlooks.md</t>
+          <t>scraped_markdown/automotiveworld/markets.md</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>72</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>The page is about automotive markets, production trends, and demand, which is related to automotive supply chains and EV manufacturing context.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/oems/</t>
+          <t>https://www.automotiveworld.com/news/</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-04-01T07:50:42+00:00</t>
+          <t>2026-04-01T09:01:45+00:00</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/oems.md</t>
+          <t>scraped_markdown/automotiveworld/news.md</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>78</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Automotive industry news page likely includes EV manufacturing and supply chain coverage.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/data/sales/</t>
+          <t>https://www.automotiveworld.com/data/oem-outlooks/</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-03-31T15:32:04+00:00</t>
+          <t>2026-03-30T13:13:27+00:00</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/sales.md</t>
+          <t>scraped_markdown/automotiveworld/oem-outlooks.md</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>82</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Contains OEM production data and automaker forecasts, which relate to automotive manufacturing and supply chains.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/software-defined-vehicle/</t>
+          <t>https://www.automotiveworld.com/topics/oems/</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-04-01T07:38:01+00:00</t>
+          <t>2026-04-01T09:01:45+00:00</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/software-defined-vehicle.md</t>
+          <t>scraped_markdown/automotiveworld/oems.md</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
           <t>success</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>68</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>OEM articles are relevant to vehicle manufacturing and likely automotive supply chains.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
+          <t>https://www.automotiveworld.com/data/sales/</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-03-31T15:32:04+00:00</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>scraped_markdown/automotiveworld/sales.md</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>41</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>This page is about OEM sales data and forecasts, not EV manufacturing or supply chains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>https://www.automotiveworld.com/topics/software-defined-vehicle/</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-04-01T09:01:45+00:00</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>scraped_markdown/automotiveworld/software-defined-vehicle.md</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>31</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Content is about software-defined vehicles, not specifically EV manufacturing or automotive supply chains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
           <t>https://www.automotiveworld.com/file-tag/data/</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B153" t="inlineStr">
         <is>
           <t>2026-03-31T09:35:12+00:00</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>scraped_markdown/automotiveworld/data_151.md</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>success</t>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>scraped_markdown/automotiveworld/data_153.md</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>12</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Only an archive date list is shown, with no article content about EV manufacturing or supply chains.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new articles and updates for MotorTrend, enhance markdown processing, and implement pipeline runner service
- Created new markdown files for articles on the Nissan Pathfinder, SUVs under $50k and $70k, and Hyundai Boulder.
- Added a comprehensive overview of MotorTrend's offerings and a yearlong review of the BMW M2.
- Improved final markdown service to validate markdown content and prevent disallowed prose.
- Introduced a new pipeline runner service to manage site processing and generate flow diagrams.
</commit_message>
<xml_diff>
--- a/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
+++ b/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The body is mostly a teaser and subscription prompt, with no substantive engineering content or technical analysis.</t>
+          <t>Body is just a teaser with no substantive engineering content beyond a generic mention of hybrids and EV plans.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The body is a legal/corporate governance story with no substantive engineering, validation, or vehicle technology content.</t>
+          <t>Body is mainly corporate litigation and judicial recusal around Musk/Tesla, with no substantive automotive engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -576,13 +576,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Body discusses Cybercab production architecture, unsupervised autonomy readiness, regulatory constraints, and program leadership impacts relevant to automotive engineering.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>Body contains substantive engineering and validation implications around Cybercab production, driverless autonomy readiness, regulatory constraints, and program leadership churn.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -617,13 +621,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The body covers fuel-cell unit cell development, control elements, and heavy-duty hydrogen architecture, which is directly relevant to engineering teams.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>Body includes concrete fuel-cell architecture and control development for heavy-duty transport, which is relevant engineering R&amp;D.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -649,7 +657,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -658,7 +666,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Mostly financial restructuring and production-location news; it mentions SPA2 and Charleston consolidation but gives little engineering or validation substance.</t>
+          <t>Body is mainly financial restructuring and production-location consolidation, with only brief mention of SPA2 shared platform and manufacturing implications.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -690,7 +698,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -699,7 +707,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Body contains concrete paint-shop energy, booth recirculation, digital printing, and robot application technology with engineering and process-efficiency implications.</t>
+          <t>Body contains concrete paint-shop engineering details on energy integration, air recirculation, digital printing, and robot geometry affecting manufacturing design and efficiency.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -735,7 +743,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -744,7 +752,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Body is a purchase-order and fleet-capacity announcement with no engineering detail beyond basic production and deployment claims.</t>
+          <t>Mostly a fleet order/partnership announcement with production and deployment counts, not engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -776,7 +784,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -785,7 +793,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Mostly plant output, demand, and market/writedown coverage; the body has no real engineering or R&amp;D substance.</t>
+          <t>Mostly plant-capacity and demand commentary; the body has no substantive engineering or R&amp;D detail beyond production scheduling.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -826,7 +834,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Body is just an award announcement with no engineering, validation, or technical substance.</t>
+          <t>Body is just an award announcement with no engineering or R&amp;D detail, only design recognition and voting context.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -858,22 +866,26 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Mentions adaptation to Tokyo road conditions and a safety validation layer, but the body is mostly a rollout/status update with limited engineering detail.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>The body discusses autonomous system adaptation to Tokyo roads, supervised operations, and safety validation architecture, which is useful engineering context.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -899,7 +911,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -908,13 +920,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The body discusses fuel-cell system R&amp;D, unit-cell expertise, cost/efficiency improvements, and heavy-vehicle application engineering.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>Body discusses fuel cell system development, cost, efficiency, and heavy-vehicle application strategy, which is directly relevant to automotive engineering.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -940,7 +956,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -949,7 +965,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Body is a short sales forecast snippet about regional demand, not engineering or R&amp;D content.</t>
+          <t>Body is just a sales forecast summary with no engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -990,7 +1006,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Mentions R&amp;D and ADAS targets, but the body is mainly a corporate sales/ROI plan with little engineering detail.</t>
+          <t>Contains some R&amp;D and ADAS/electrification investment targets, but the body is mostly corporate financial planning and manufacturing strategy without engineering detail.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1022,7 +1038,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1031,7 +1047,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Mostly a corporate milestone and portfolio announcement, with only brief mention of a battery facility and future BEV models, not substantive engineering detail.</t>
+          <t>Mostly a corporate milestone and portfolio/planning update; the body gives little engineering detail beyond a new battery facility and future BEV models.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1063,7 +1079,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1072,7 +1088,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>It discusses HDV emissions policy and charging rollout, but the body is regulatory compliance rather than engineering or R&amp;D detail.</t>
+          <t>This is mainly a regulatory policy update with no substantive engineering, validation, or vehicle development detail in the body.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1104,22 +1120,26 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Mostly a product launch with specs and rollout plans; the body gives only light ADAS/validation detail and little substantive engineering analysis.</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
+          <t>The body contains real engineering content on a new platform, ADAS architecture, Qualcomm/LiDAR setup, OTA rollout, battery fast-charging, and validation testing.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1174,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Body is only a short production blurb plus a paywall prompt, with no engineering or R&amp;D substance.</t>
+          <t>Body contains only a brief production statistic and a paywall prompt, with no engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -1186,7 +1206,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1195,7 +1215,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Mostly a showcase/launch blurb with limited engineering detail beyond swappable batteries and SDV mention.</t>
+          <t>Mentions a few engineering features, but the body is mostly a product/showcase promo with little technical depth or validation detail.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1227,7 +1247,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1236,7 +1256,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Mostly a plant anniversary and investment/news item with vehicle premieres and sales context, but no substantive engineering, validation, or technical development detail.</t>
+          <t>Body is mainly a plant-anniversary and model-premiere announcement with investment and sales context, not engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -1268,7 +1288,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1277,7 +1297,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Mostly a model-range/event announcement with pricing and trims; no substantive engineering or validation detail in the body.</t>
+          <t>Mostly a product/market announcement about new PV5 variants and pricing, with little engineering depth beyond body-length and conversion compatibility.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1318,7 +1338,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Body is mainly a service launch and deployment announcement, with no substantive engineering, validation, or architecture detail.</t>
+          <t>Mostly a commercial rollout announcement with launch locations, permits, and ownership details; the body gives little engineering or validation substance.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1350,7 +1370,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1359,13 +1379,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>The body has substantive engineering detail on a unified truck software architecture, ECU hardware testing, OTA updates, and modular compute consolidation.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>Describes a unified truck software architecture, ECU/hardware integration timing, OTA updates, and compute consolidation—clear engineering relevance.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1424,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>The body is mainly a consumer infotainment rollout with platform branding and content delivery, not substantive automotive engineering or validation detail.</t>
+          <t>Body is mainly a consumer entertainment platform launch with little engineering depth beyond Android Automotive and personalization.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1441,13 +1465,17 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>The body describes a real LiDAR/edge-AI intersection sensing platform, with FMCW 4D sensor operation and safety/traffic monitoring implications relevant to engineering teams.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
+          <t>Body gives concrete LiDAR/edge-AI intersection sensing details, deployment scope, and safety applications relevant to engineering and validation.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1501,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1482,7 +1510,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>The body discusses a fleet-wide robotaxi software/network failure, emergency systems, fail-safe behavior, and safety/validation implications.</t>
+          <t>Body gives concrete engineering relevance: fleet-wide software/network failure, emergency fallback breakdown, and autonomous safety/validation risks.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1518,7 +1546,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1527,13 +1555,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>The body gives concrete engineering detail on digital key standards, interoperability, validation, and tradeoffs in security, reliability, and power management.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
+          <t>The body discusses digital key architecture, interoperability, security, testing, and integration effort, which are directly relevant to automotive software and validation work.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1591,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1568,13 +1600,17 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Body gives concrete autonomy integration, sensor suite, powertrain, safety-driver, and real-route validation details relevant to engineering and deployment.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>Real-world autonomous truck pilot with factory-integrated sensors, powertrain, safety-driver supervision, and validation of uptime, serviceability, and route operations.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1636,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1609,7 +1645,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Mostly a service launch and operations update, with little engineering detail beyond naming the AV models and training.</t>
+          <t>Mostly a service launch and rollout update; the body gives little engineering detail beyond named AV models and operations/training.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1641,7 +1677,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1650,7 +1686,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Mostly a corporate integration announcement; the body gives only high-level references to shared development and zero-emission tech without engineering detail.</t>
+          <t>Mostly a corporate integration announcement; the body only briefly mentions shared development and zero-emission technologies without technical engineering detail.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1682,7 +1718,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1691,7 +1727,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Body is a consumer app-access partnership with CarPlay/Android Auto integration, not substantive vehicle engineering or R&amp;D content.</t>
+          <t>Body is mainly a consumer app-perk announcement with CarPlay/Android Auto integration, not engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1723,22 +1759,22 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>The body discusses battery chemistry, production scale-up, subsidies, supply-chain risk, and manufacturing challenges that matter to automotive R&amp;D and platform planning.</t>
+          <t>Body is mainly policy and investment strategy, with only brief battery-supply context and little engineering or validation detail.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -1764,22 +1800,26 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Body has a real powertrain engineering concept and testing detail, but it is mainly a product/test announcement with little technical depth or validation substance.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+          <t>Body gives concrete engineering detail on HPDI hydrogen combustion architecture, efficiency, power, and commercial validation testing.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1845,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1814,7 +1854,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>The body gives concrete drivetrain, actuator, and control-platform details about a new torque-vectoring architecture with real-time vehicle dynamics implications.</t>
+          <t>Body gives concrete drivetrain and control-architecture details on electromechanical rear-axle torque vectoring, actuator behavior, and real-time vehicle dynamics integration.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1859,7 +1899,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>The body gives concrete ADAS engineering and validation failures in BlueCruise, including driver monitoring, braking behavior, speed limits, and data recording gaps.</t>
+          <t>The body gives concrete ADAS engineering and validation failures—driver monitoring, braking behavior, speed limits, and missing data standards—directly relevant to R&amp;D and safety work.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1895,7 +1935,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1904,7 +1944,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Mostly a partnership and financing announcement with only high-level claims about purpose-built autonomous EVs, with no substantive engineering detail or validation content.</t>
+          <t>Mostly a partnership and financing announcement, with only brief high-level mention of purpose-built autonomous small EVs and no real engineering detail.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -1936,7 +1976,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1945,7 +1985,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Body gives a useful EV thermal architecture summary, but it is mostly a supplier product description with limited engineering depth or validation detail.</t>
+          <t>The body gives a high-level integration summary of an EV thermal module, but little engineering depth beyond component listing and claimed packaging/range benefits.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -1986,7 +2026,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Body discusses a safety-certified RTOS used in AI domain controller platforms, with ISO 26262, deterministic execution, and cockpit-ADAS fusion architecture details.</t>
+          <t>The body discusses a pre-certified RTOS used in AI domain controller platforms, with ISO 26262, deterministic execution, and cockpit-ADAS fusion architecture implications.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2022,7 +2062,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2031,7 +2071,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Mostly manufacturing economics and tariff strategy; the body gives little engineering detail beyond where models are built and production timing.</t>
+          <t>Body is mainly about pricing, tariffs, and manufacturing location economics, with little engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -2063,7 +2103,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2072,17 +2112,13 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Body describes live V2X interoperability testing between vehicle OBU and roadside units, with deployment implications for OEM and aftermarket systems.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body describes live V2X tolling interoperability testing, OBU/RSU communication, and retrofit deployment implications, which are useful engineering details.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2144,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2117,7 +2153,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Primarily a production-network and investment announcement, with little engineering or R&amp;D substance beyond generic mention of drivetrains and future cab generations.</t>
+          <t>Mostly a production-network and investment announcement; the body lacks substantive engineering or R&amp;D detail beyond generic assembly and complexity management.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -2149,7 +2185,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2158,17 +2194,13 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Body gives concrete engineering use cases for HMI, ADAS scenario verification, and LiDAR point cloud simulation with a game-engine-based industrial 3D engine.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body describes an engineering tool for cockpit HMI, ADAS verification, and LiDAR point-cloud simulation, with implications for development and validation workflows.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2226,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2203,7 +2235,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>This is a sales forecast and market outlook with no engineering or R&amp;D substance in the body.</t>
+          <t>Body is a sales-market forecast with macro demand and pricing factors, not engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -2235,7 +2267,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2244,7 +2276,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Mostly a product announcement with range, trims, and sales timing; little engineering or R&amp;D substance beyond basic platform and charging specs.</t>
+          <t>Mostly a product announcement with specs and trim details; little engineering depth or R&amp;D insight beyond platform and range figures.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -2276,7 +2308,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2285,7 +2317,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Mostly a product launch with trim, display, and launch timing details; the body gives little engineering depth beyond basic hybrid and e-AWD mention.</t>
+          <t>Mostly a product announcement with specs and features; little engineering depth beyond a brief hybrid/e-AWD mention.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -2317,7 +2349,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2326,7 +2358,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>This is an editorial calendar/listing page with dates and link titles, not substantive engineering or R&amp;D narrative.</t>
+          <t>This is an editorial calendar/listing page with dates and article links, not substantive engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
@@ -2399,7 +2431,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2408,7 +2440,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Paywalled login/subscribe page with no article narrative or engineering content in the body.</t>
+          <t>No article body is present; this is only a subscription/login gate with no engineering content.</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -2941,7 +2973,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>This is just an archive/listing of dates with no substantive article narrative or engineering content.</t>
+          <t>Body is just a date list/archive page with no article narrative or engineering content.</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>

</xml_diff>

<commit_message>
Refactor motortrend_final.md for clarity and detail; add 403 error handling in sitemap_nodes.py; update pipeline_runner_service.py to save flow diagrams as PNG; remove obsolete Mermaid diagram files and generate new ones.
</commit_message>
<xml_diff>
--- a/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
+++ b/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -494,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Body is just a teaser with no substantive engineering content beyond a generic mention of hybrids and EV plans.</t>
+          <t>Body is just a brief teaser plus subscription prompt, with no substantive engineering analysis.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Body is mainly corporate litigation and judicial recusal around Musk/Tesla, with no substantive automotive engineering or R&amp;D content.</t>
+          <t>The body is a legal/corporate governance dispute about Musk and Delaware courts, with no substantive automotive engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -576,7 +576,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Body contains substantive engineering and validation implications around Cybercab production, driverless autonomy readiness, regulatory constraints, and program leadership churn.</t>
+          <t>Body has substantive engineering and validation implications around Cybercab production readiness, unsupervised autonomy risk, and regulatory constraints on a no-controls vehicle.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Body includes concrete fuel-cell architecture and control development for heavy-duty transport, which is relevant engineering R&amp;D.</t>
+          <t>The body describes a concrete fuel-cell engineering collaboration on unit cells, architecture, and control elements for heavy-duty transport.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Body is mainly financial restructuring and production-location consolidation, with only brief mention of SPA2 shared platform and manufacturing implications.</t>
+          <t>Mostly financial restructuring and production-location news; the body lacks substantive engineering or validation detail beyond a brief SPA2/assembly mention.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Body contains concrete paint-shop engineering details on energy integration, air recirculation, digital printing, and robot geometry affecting manufacturing design and efficiency.</t>
+          <t>Contains substantive paint-shop engineering details on energy recovery, modular booth design, digital printing, and robot geometry relevant to manufacturing R&amp;D.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Mostly a fleet order/partnership announcement with production and deployment counts, not engineering or R&amp;D substance.</t>
+          <t>Body is mainly an order/customer announcement with fleet and production figures, not engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Mostly plant-capacity and demand commentary; the body has no substantive engineering or R&amp;D detail beyond production scheduling.</t>
+          <t>Primarily production and demand news about plant shifts and layoffs, with no substantive engineering, validation, or technical development detail.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -834,7 +834,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Body is just an award announcement with no engineering or R&amp;D detail, only design recognition and voting context.</t>
+          <t>Body is mainly an award announcement with no engineering, validation, or technical detail.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -866,26 +866,22 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The body discusses autonomous system adaptation to Tokyo roads, supervised operations, and safety validation architecture, which is useful engineering context.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Contains some engineering content on adapting autonomous driving and safety validation, but it is mostly a rollout/partnership update with limited technical depth.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -911,7 +907,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -920,7 +916,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Body discusses fuel cell system development, cost, efficiency, and heavy-vehicle application strategy, which is directly relevant to automotive engineering.</t>
+          <t>Discusses fuel cell system development, cost, efficiency, and heavy-duty engineering scale, which is relevant to automotive R&amp;D.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -965,7 +961,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Body is just a sales forecast summary with no engineering or R&amp;D substance.</t>
+          <t>Body is a brief sales forecast snippet with market demand figures, not engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -997,7 +993,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1006,7 +1002,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Contains some R&amp;D and ADAS/electrification investment targets, but the body is mostly corporate financial planning and manufacturing strategy without engineering detail.</t>
+          <t>Contains some R&amp;D and ADAS/electrification planning, but the body is mostly financial targets and corporate strategy rather than engineering detail.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1047,7 +1043,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Mostly a corporate milestone and portfolio/planning update; the body gives little engineering detail beyond a new battery facility and future BEV models.</t>
+          <t>Mostly corporate history and production news with only brief mention of BEV models and a battery plant, but no real engineering or validation detail.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1079,7 +1075,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1088,7 +1084,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>This is mainly a regulatory policy update with no substantive engineering, validation, or vehicle development detail in the body.</t>
+          <t>Mostly policy/compliance news about CO2 targets and credits, with no substantive engineering or vehicle development detail in the body.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1120,26 +1116,22 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>The body contains real engineering content on a new platform, ADAS architecture, Qualcomm/LiDAR setup, OTA rollout, battery fast-charging, and validation testing.</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Contains some engineering details on platform, ADAS, LiDAR, battery and validation, but it is mainly a product launch announcement with limited technical depth.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1157,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1174,7 +1166,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Body contains only a brief production statistic and a paywall prompt, with no engineering or R&amp;D substance.</t>
+          <t>Body is just a production summary with a paywall stub, offering no substantive engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -1206,7 +1198,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1215,7 +1207,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Mentions a few engineering features, but the body is mostly a product/showcase promo with little technical depth or validation detail.</t>
+          <t>Mentions some engineering elements like pedal-by-wire, swappable batteries, regen and SDV, but the body is mostly a product/showcase announcement with little technical depth.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1247,7 +1239,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1256,7 +1248,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Body is mainly a plant-anniversary and model-premiere announcement with investment and sales context, not engineering or R&amp;D detail.</t>
+          <t>Body is mainly a plant anniversary and vehicle premiere announcement with investment and sales context, not engineering detail.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -1297,7 +1289,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Mostly a product/market announcement about new PV5 variants and pricing, with little engineering depth beyond body-length and conversion compatibility.</t>
+          <t>Mostly a product debut and pricing announcement with only brief mention of platform variants and conversions, not substantive engineering detail.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1329,7 +1321,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1338,7 +1330,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mostly a commercial rollout announcement with launch locations, permits, and ownership details; the body gives little engineering or validation substance.</t>
+          <t>Mostly a commercial rollout and partnership announcement with no substantive engineering, architecture, or validation detail in the body.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1370,7 +1362,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1379,7 +1371,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Describes a unified truck software architecture, ECU/hardware integration timing, OTA updates, and compute consolidation—clear engineering relevance.</t>
+          <t>Describes a unified truck software platform with EE architecture, HPCs, ECU integration timing, OTA updates, and modular compute design.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1415,7 +1407,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1424,7 +1416,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Body is mainly a consumer entertainment platform launch with little engineering depth beyond Android Automotive and personalization.</t>
+          <t>It describes an infotainment/media platform and content delivery, but offers little engineering detail beyond standard Android Automotive integration.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1465,7 +1457,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Body gives concrete LiDAR/edge-AI intersection sensing details, deployment scope, and safety applications relevant to engineering and validation.</t>
+          <t>The body has concrete engineering detail on FMCW 4D LiDAR, edge AI perception, and intersection safety/traffic monitoring deployment, which is useful for transportation/ADAS-style systems work.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1501,7 +1493,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1510,7 +1502,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Body gives concrete engineering relevance: fleet-wide software/network failure, emergency fallback breakdown, and autonomous safety/validation risks.</t>
+          <t>The body gives concrete engineering relevance: a fleet-wide system fault, failed SOS/customer infrastructure, and safety/operational implications for autonomous vehicle validation and fail-safe design.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1555,17 +1547,13 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>The body discusses digital key architecture, interoperability, security, testing, and integration effort, which are directly relevant to automotive software and validation work.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body discusses digital key architecture, interoperability, security, reliability, and integration/testing trade-offs that directly affect vehicle software and validation work.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1579,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1600,7 +1588,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Real-world autonomous truck pilot with factory-integrated sensors, powertrain, safety-driver supervision, and validation of uptime, serviceability, and route operations.</t>
+          <t>Body gives concrete autonomous-truck engineering and validation details: factory-integrated sensors/software, live freight route, route coverage, serviceability, and operational data collection.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1636,7 +1624,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1645,7 +1633,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Mostly a service launch and rollout update; the body gives little engineering detail beyond named AV models and operations/training.</t>
+          <t>Body is mainly a service launch and rollout update with minimal engineering detail beyond generic AV operations and training.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1677,7 +1665,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1686,7 +1674,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Mostly a corporate integration announcement; the body only briefly mentions shared development and zero-emission technologies without technical engineering detail.</t>
+          <t>The body is mostly a corporate integration announcement with only brief, high-level mentions of shared development and zero-emission technologies, without engineering detail.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1718,7 +1706,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1727,7 +1715,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Body is mainly a consumer app-perk announcement with CarPlay/Android Auto integration, not engineering or R&amp;D detail.</t>
+          <t>Mostly a consumer app partnership and personalization promo, with no substantive engineering, validation, or platform detail in the body.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1759,7 +1747,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1768,7 +1756,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Body is mainly policy and investment strategy, with only brief battery-supply context and little engineering or validation detail.</t>
+          <t>Body is mainly industrial policy and battery investment news; it mentions solid-state batteries and supply-chain risk, but little engineering detail or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1800,7 +1788,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1809,17 +1797,13 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Body gives concrete engineering detail on HPDI hydrogen combustion architecture, efficiency, power, and commercial validation testing.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body gives concrete engineering detail on HPDI hydrogen combustion testing, power/efficiency tradeoffs, and powertrain strategy, which is useful for automotive R&amp;D.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1829,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1854,7 +1838,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Body gives concrete drivetrain and control-architecture details on electromechanical rear-axle torque vectoring, actuator behavior, and real-time vehicle dynamics integration.</t>
+          <t>Body has concrete drivetrain and control architecture details, including rear-axle electromechanical torque vectoring, 400V actuator, and real-time vehicle dynamics integration.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1890,7 +1874,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1899,7 +1883,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>The body gives concrete ADAS engineering and validation failures—driver monitoring, braking behavior, speed limits, and missing data standards—directly relevant to R&amp;D and safety work.</t>
+          <t>The body gives concrete ADAS failure modes, driver monitoring gaps, and regulatory implications that are directly useful to automotive validation and safety engineering.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1935,7 +1919,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1944,7 +1928,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Mostly a partnership and financing announcement, with only brief high-level mention of purpose-built autonomous small EVs and no real engineering detail.</t>
+          <t>Body is mostly a partnership/funding announcement with only broad claims about purpose-built autonomous EVs, not substantive engineering or validation detail.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -1976,22 +1960,26 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>The body gives a high-level integration summary of an EV thermal module, but little engineering depth beyond component listing and claimed packaging/range benefits.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
+          <t>The body describes an integrated EV thermal management architecture and its engineering benefits for charging, performance, packaging, and energy use.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2014,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>The body discusses a pre-certified RTOS used in AI domain controller platforms, with ISO 26262, deterministic execution, and cockpit-ADAS fusion architecture implications.</t>
+          <t>Discusses a safety-certified RTOS architecture for AI/domain controllers with ISO 26262, deterministic execution, and cockpit-ADAS fusion implications.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2062,7 +2050,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2071,7 +2059,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Body is mainly about pricing, tariffs, and manufacturing location economics, with little engineering or R&amp;D detail.</t>
+          <t>Mostly trade and manufacturing-cost discussion; no substantive engineering or R&amp;D detail beyond where Nissan chooses to build models.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -2112,13 +2100,17 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>The body describes live V2X tolling interoperability testing, OBU/RSU communication, and retrofit deployment implications, which are useful engineering details.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
+          <t>Body describes live V2X interoperability testing with OBU/RSU architecture and aftermarket deployment implications, which is useful engineering validation content.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2136,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2153,7 +2145,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Mostly a production-network and investment announcement; the body lacks substantive engineering or R&amp;D detail beyond generic assembly and complexity management.</t>
+          <t>Mainly a production-network and cost-optimization announcement, with no substantive engineering or R&amp;D detail beyond generic assembly planning.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -2185,7 +2177,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2194,7 +2186,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>The body describes an engineering tool for cockpit HMI, ADAS verification, and LiDAR point-cloud simulation, with implications for development and validation workflows.</t>
+          <t>The body describes a real-time 3D engine for cockpit HMI, ADAS scenario verification, and digital twin simulation, with engineering workflow and simulator details.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -2226,7 +2218,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2235,7 +2227,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Body is a sales-market forecast with macro demand and pricing factors, not engineering or R&amp;D substance.</t>
+          <t>This is a market sales forecast with regional demand and macroeconomic factors, not engineering or R&amp;D content.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -2267,7 +2259,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2276,7 +2268,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Mostly a product announcement with specs and trim details; little engineering depth or R&amp;D insight beyond platform and range figures.</t>
+          <t>Mostly a product announcement with specs and launch timing; the body lacks substantive engineering or R&amp;D analysis.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -2308,7 +2300,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2317,7 +2309,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Mostly a product announcement with specs and features; little engineering depth beyond a brief hybrid/e-AWD mention.</t>
+          <t>Mostly a vehicle launch/update with basic powertrain and feature specs, not substantive engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -2358,7 +2350,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>This is an editorial calendar/listing page with dates and article links, not substantive engineering or R&amp;D content.</t>
+          <t>This is an editorial calendar/listing page with dates and article links, not substantive engineering content.</t>
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
@@ -2431,7 +2423,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2440,7 +2432,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>No article body is present; this is only a subscription/login gate with no engineering content.</t>
+          <t>Subscription/login gate with no article narrative or engineering content in the body.</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -2973,7 +2965,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Body is just a date list/archive page with no article narrative or engineering content.</t>
+          <t>Body is just a date-based archive list with no article narrative or engineering content.</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: add HTML report generation service with markdown parsing and rendering
</commit_message>
<xml_diff>
--- a/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
+++ b/extracted_urls/automotiveworld/automotiveworld_urls.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -494,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Body is just a brief teaser plus subscription prompt, with no substantive engineering analysis.</t>
+          <t>Body is just a teaser and subscription gate with no substantive engineering analysis.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The body is a legal/corporate governance dispute about Musk and Delaware courts, with no substantive automotive engineering or R&amp;D content.</t>
+          <t>Mostly corporate litigation and governance about Musk/Tesla, with no substantive engineering, validation, or R&amp;D detail in the body.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -576,17 +576,13 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Body has substantive engineering and validation implications around Cybercab production readiness, unsupervised autonomy risk, and regulatory constraints on a no-controls vehicle.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body contains substantive engineering and validation implications for a driverless vehicle platform, including autonomy readiness, crash performance, regulatory constraints, and production ramp risk.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -612,7 +608,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -621,17 +617,13 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The body describes a concrete fuel-cell engineering collaboration on unit cells, architecture, and control elements for heavy-duty transport.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body covers fuel-cell system development, unit-cell production, and architecture/control elements for heavy-duty applications, which is relevant engineering content.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -657,7 +649,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -666,7 +658,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Mostly financial restructuring and production-location news; the body lacks substantive engineering or validation detail beyond a brief SPA2/assembly mention.</t>
+          <t>Body is mainly about debt restructuring and production consolidation, with only brief mention of SPA2 and manufacturing location.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -698,26 +690,22 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Contains substantive paint-shop engineering details on energy recovery, modular booth design, digital printing, and robot geometry relevant to manufacturing R&amp;D.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body has some engineering content on paint-shop energy, digital printing, and robot geometry, but it is mainly a product showcase/event promotion with limited R&amp;D depth.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -752,7 +740,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Body is mainly an order/customer announcement with fleet and production figures, not engineering or R&amp;D substance.</t>
+          <t>Mostly a fleet order and company production update, with no substantive engineering, validation, or architecture detail in the body.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -784,7 +772,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -793,7 +781,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Primarily production and demand news about plant shifts and layoffs, with no substantive engineering, validation, or technical development detail.</t>
+          <t>Body is mainly production, sales, and demand shift reporting with no real engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -825,7 +813,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -834,7 +822,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Body is mainly an award announcement with no engineering, validation, or technical detail.</t>
+          <t>Body is just an award announcement with no engineering or technical substance.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -866,22 +854,22 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Contains some engineering content on adapting autonomous driving and safety validation, but it is mostly a rollout/partnership update with limited technical depth.</t>
+          <t>Describes autonomous system adaptation to Tokyo roads and mentions safety validation architecture, which is relevant engineering context.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -907,26 +895,22 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Discusses fuel cell system development, cost, efficiency, and heavy-duty engineering scale, which is relevant to automotive R&amp;D.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body has some fuel-cell R&amp;D and cost/efficiency discussion, but it is mainly a partnership/strategy piece rather than substantive engineering detail.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -952,7 +936,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -961,7 +945,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Body is a brief sales forecast snippet with market demand figures, not engineering or R&amp;D content.</t>
+          <t>Body is a brief sales-demand snapshot with no engineering, validation, or technical substance.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -993,7 +977,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1002,7 +986,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Contains some R&amp;D and ADAS/electrification planning, but the body is mostly financial targets and corporate strategy rather than engineering detail.</t>
+          <t>Mostly a corporate strategy and sales-target announcement; the body only briefly mentions R&amp;D spend, electrification, and ADAS with no engineering detail.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1034,7 +1018,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1043,7 +1027,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Mostly corporate history and production news with only brief mention of BEV models and a battery plant, but no real engineering or validation detail.</t>
+          <t>Mostly business milestone and portfolio news, with only brief mention of a battery facility and new BEV models, but no substantive engineering detail.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1075,7 +1059,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1084,7 +1068,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Mostly policy/compliance news about CO2 targets and credits, with no substantive engineering or vehicle development detail in the body.</t>
+          <t>Policy update on HDV CO2 credits and targets, with no substantive engineering, validation, or technical development content.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1116,7 +1100,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1125,7 +1109,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Contains some engineering details on platform, ADAS, LiDAR, battery and validation, but it is mainly a product launch announcement with limited technical depth.</t>
+          <t>Contains some ADAS and platform details, but the body is mainly a product launch with specs and rollout plans rather than deep engineering or validation substance.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -1157,7 +1141,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1166,7 +1150,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Body is just a production summary with a paywall stub, offering no substantive engineering or R&amp;D content.</t>
+          <t>Body is just a brief production statistic and paywall teaser, with no engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -1198,7 +1182,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1207,7 +1191,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Mentions some engineering elements like pedal-by-wire, swappable batteries, regen and SDV, but the body is mostly a product/showcase announcement with little technical depth.</t>
+          <t>Body is mostly a product showcase for a micromobility vehicle, with only brief engineering details and no substantive R&amp;D or validation depth.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1248,7 +1232,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Body is mainly a plant anniversary and vehicle premiere announcement with investment and sales context, not engineering detail.</t>
+          <t>Body is mainly a plant anniversary, premieres, and investment/jobs news with no real engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -1280,7 +1264,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1289,7 +1273,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Mostly a product debut and pricing announcement with only brief mention of platform variants and conversions, not substantive engineering detail.</t>
+          <t>Mostly a product debut and pricing note with no substantive engineering or validation detail in the body.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1321,7 +1305,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1330,7 +1314,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mostly a commercial rollout and partnership announcement with no substantive engineering, architecture, or validation detail in the body.</t>
+          <t>Commercial robotaxi launch announcement with regulatory and rollout details, but little engineering or validation substance in the body.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1362,7 +1346,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1371,17 +1355,13 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Describes a unified truck software platform with EE architecture, HPCs, ECU integration timing, OTA updates, and modular compute design.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>The body describes a unified software-defined vehicle architecture, ECU testing timeline, multi-chipset middleware, OTA updates, and compute consolidation, all directly relevant to automotive EE and software engineering.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1387,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1416,7 +1396,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>It describes an infotainment/media platform and content delivery, but offers little engineering detail beyond standard Android Automotive integration.</t>
+          <t>Mostly a consumer infotainment rollout with no substantive engineering, validation, or architecture detail beyond platform branding and content delivery.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1448,26 +1428,22 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>selected</t>
+          <t>not_selected</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>The body has concrete engineering detail on FMCW 4D LiDAR, edge AI perception, and intersection safety/traffic monitoring deployment, which is useful for transportation/ADAS-style systems work.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body has some engineering substance on FMCW 4D LiDAR intersection sensing, but it is mainly an infrastructure deployment announcement rather than automotive R&amp;D-focused work.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>skipped_not_selected</t>
         </is>
       </c>
     </row>
@@ -1502,17 +1478,13 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>The body gives concrete engineering relevance: a fleet-wide system fault, failed SOS/customer infrastructure, and safety/operational implications for autonomous vehicle validation and fail-safe design.</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
-        </is>
-      </c>
+          <t>Body describes a fleet-wide robotaxi software/network fault, emergency-system failure, and safety/validation risks that are directly relevant to autonomous vehicle engineering.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>appended</t>
+          <t>error</t>
         </is>
       </c>
     </row>
@@ -1547,13 +1519,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Body discusses digital key architecture, interoperability, security, reliability, and integration/testing trade-offs that directly affect vehicle software and validation work.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
+          <t>Focuses on digital key architecture, interoperability, security, and validation trade-offs, with concrete integration and testing detail.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1555,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1588,7 +1564,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Body gives concrete autonomous-truck engineering and validation details: factory-integrated sensors/software, live freight route, route coverage, serviceability, and operational data collection.</t>
+          <t>Live autonomous truck pilot with factory-integrated sensors, powertrain, software, and validation goals on a real freight route.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1624,7 +1600,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1633,7 +1609,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Body is mainly a service launch and rollout update with minimal engineering detail beyond generic AV operations and training.</t>
+          <t>Contains some autonomous vehicle deployment details, but the body is mainly a service launch and operations update with little engineering depth.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1665,7 +1641,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1674,7 +1650,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>The body is mostly a corporate integration announcement with only brief, high-level mentions of shared development and zero-emission technologies, without engineering detail.</t>
+          <t>Mostly a corporate holding-company launch and ownership update; the body only briefly mentions shared development and zero-emission themes without engineering detail.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1706,7 +1682,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1715,7 +1691,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Mostly a consumer app partnership and personalization promo, with no substantive engineering, validation, or platform detail in the body.</t>
+          <t>Mostly a promotional app-access partnership with no substantive engineering, validation, or vehicle architecture detail in the body.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1747,7 +1723,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1756,7 +1732,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Body is mainly industrial policy and battery investment news; it mentions solid-state batteries and supply-chain risk, but little engineering detail or R&amp;D substance.</t>
+          <t>Body is mainly policy and investment strategy; it mentions battery scale and solid-state chemistry but gives little engineering or validation detail.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1797,13 +1773,17 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Body gives concrete engineering detail on HPDI hydrogen combustion testing, power/efficiency tradeoffs, and powertrain strategy, which is useful for automotive R&amp;D.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+          <t>Body discusses an on-road tested hydrogen HPDI powertrain and its efficiency, range, and ZEV engineering implications.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1809,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1838,7 +1818,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Body has concrete drivetrain and control architecture details, including rear-axle electromechanical torque vectoring, 400V actuator, and real-time vehicle dynamics integration.</t>
+          <t>Describes a real production torque-vectoring architecture, control integration, and operating behavior with clear vehicle-dynamics engineering detail.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1874,7 +1854,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1883,7 +1863,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>The body gives concrete ADAS failure modes, driver monitoring gaps, and regulatory implications that are directly useful to automotive validation and safety engineering.</t>
+          <t>The body gives concrete ADAS safety and validation failures, driver monitoring issues, and regulatory implications directly relevant to automotive engineering.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1919,7 +1899,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1928,7 +1908,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Body is mostly a partnership/funding announcement with only broad claims about purpose-built autonomous EVs, not substantive engineering or validation detail.</t>
+          <t>Body is mostly a partnership/financing announcement with only brief, high-level vehicle-purpose claims and no engineering detail.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -1960,7 +1940,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1969,7 +1949,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>The body describes an integrated EV thermal management architecture and its engineering benefits for charging, performance, packaging, and energy use.</t>
+          <t>The body describes an integrated EV thermal management architecture and its impact on packaging, complexity, charging, and energy use.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2005,7 +1985,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2014,7 +1994,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Discusses a safety-certified RTOS architecture for AI/domain controllers with ISO 26262, deterministic execution, and cockpit-ADAS fusion implications.</t>
+          <t>Body gives concrete engineering detail on safety-certified RTOS integration, ISO 26262, deterministic execution, and domain-controller architecture for cockpit-ADAS fusion.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2050,7 +2030,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2059,7 +2039,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Mostly trade and manufacturing-cost discussion; no substantive engineering or R&amp;D detail beyond where Nissan chooses to build models.</t>
+          <t>The body is mainly about tariffs, plant footprint, and pricing economics, with no substantive engineering or R&amp;D detail.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -2100,7 +2080,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Body describes live V2X interoperability testing with OBU/RSU architecture and aftermarket deployment implications, which is useful engineering validation content.</t>
+          <t>Body describes live V2X OBU/RSU interoperability testing, deployment models, and standards-based communication relevant to automotive systems engineering.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2145,7 +2125,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Mainly a production-network and cost-optimization announcement, with no substantive engineering or R&amp;D detail beyond generic assembly planning.</t>
+          <t>It is mainly a production-network and cost-optimization announcement, with little engineering or validation detail beyond general assembly-site planning.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -2177,7 +2157,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2186,13 +2166,17 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>The body describes a real-time 3D engine for cockpit HMI, ADAS scenario verification, and digital twin simulation, with engineering workflow and simulator details.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
+          <t>The body describes an engineering tool for cockpit HMI, ADAS verification, and digital twin simulation with runtime/editor architecture and a LiDAR point-cloud simulator project.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
@@ -2227,7 +2211,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>This is a market sales forecast with regional demand and macroeconomic factors, not engineering or R&amp;D content.</t>
+          <t>The body is a market sales forecast with demand and macroeconomic commentary, not engineering or R&amp;D substance.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -2259,7 +2243,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2268,7 +2252,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Mostly a product announcement with specs and launch timing; the body lacks substantive engineering or R&amp;D analysis.</t>
+          <t>Mostly a vehicle launch with specs and pricing positioning; the body lacks substantive engineering or validation detail.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -2309,7 +2293,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Mostly a vehicle launch/update with basic powertrain and feature specs, not substantive engineering or R&amp;D detail.</t>
+          <t>Mostly a product launch with specs and feature list; the body gives little engineering depth beyond announcing a hybrid and e-AWD option.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -2322,17 +2306,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/editorial-calendar/</t>
+          <t>https://www.automotiveworld.com/topics/software-defined-vehicle/faster-simpler-smarter-how-etas-busts-the-autosar-myth/</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-03-31T15:21:54+00:00</t>
+          <t>2026-04-02T06:34:35+00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/editorial-calendar.md</t>
+          <t>scraped_markdown/automotiveworld/faster-simpler-smarter-how-etas-busts-the-autosar-myth.md</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2341,39 +2325,43 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>89</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>not_selected</t>
+          <t>selected</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>This is an editorial calendar/listing page with dates and article links, not substantive engineering content.</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
+          <t>Body gives concrete engineering detail on AUTOSAR Classic tooling, ECU integration, virtual ECUs, code generation, multicore data placement, and safety/footprint tradeoffs.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>final_markdown/automotiveworld/automotiveworld_final.md</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>skipped_not_selected</t>
+          <t>appended</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/mp-files/</t>
+          <t>https://www.automotiveworld.com/editorial-calendar/</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-03-31T09:35:12+00:00</t>
+          <t>2026-03-31T15:21:54+00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/mp-files.md</t>
+          <t>scraped_markdown/automotiveworld/editorial-calendar.md</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2382,7 +2370,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2391,7 +2379,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Section landing page is dominated by listing content rather than a full article.</t>
+          <t>This is an editorial calendar/listing page with dates and links, not a substantive engineering article.</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
@@ -2404,7 +2392,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/mp-files/toyota-profile-and-production-forecast-to-2030.xlsx/</t>
+          <t>https://www.automotiveworld.com/mp-files/</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2414,7 +2402,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/toyota-profile-and-production-forecast-to-2030.xlsx.md</t>
+          <t>scraped_markdown/automotiveworld/mp-files.md</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2423,7 +2411,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2432,7 +2420,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Subscription/login gate with no article narrative or engineering content in the body.</t>
+          <t>Section landing page is dominated by listing content rather than a full article.</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -2445,17 +2433,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/analysis/</t>
+          <t>https://www.automotiveworld.com/mp-files/toyota-profile-and-production-forecast-to-2030.xlsx/</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-03-31T18:12:09+00:00</t>
+          <t>2026-03-31T09:35:12+00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/analysis.md</t>
+          <t>scraped_markdown/automotiveworld/toyota-profile-and-production-forecast-to-2030.xlsx.md</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2464,7 +2452,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2473,7 +2461,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Section landing page is dominated by listing content rather than a full article.</t>
+          <t>No article body is present; this is just a subscription/login gate with no engineering content.</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -2486,17 +2474,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/articles/</t>
+          <t>https://www.automotiveworld.com/analysis/</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-04-01T06:46:39+00:00</t>
+          <t>2026-03-31T18:12:09+00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/articles.md</t>
+          <t>scraped_markdown/automotiveworld/analysis.md</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2527,17 +2515,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/autonomous-driving/</t>
+          <t>https://www.automotiveworld.com/articles/</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-04-01T11:06:21+00:00</t>
+          <t>2026-04-01T06:46:39+00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/autonomous-driving.md</t>
+          <t>scraped_markdown/automotiveworld/articles.md</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2555,7 +2543,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Topic page is dominated by listing content and lacks substantive article narrative.</t>
+          <t>Section landing page is dominated by listing content rather than a full article.</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -2568,17 +2556,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/commercial-vehicle/</t>
+          <t>https://www.automotiveworld.com/topics/autonomous-driving/</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-04-01T14:09:18+00:00</t>
+          <t>2026-04-01T11:06:21+00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/commercial-vehicle.md</t>
+          <t>scraped_markdown/automotiveworld/autonomous-driving.md</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2609,17 +2597,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/data/</t>
+          <t>https://www.automotiveworld.com/topics/commercial-vehicle/</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-03-31T15:32:04+00:00</t>
+          <t>2026-04-01T14:09:18+00:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/data.md</t>
+          <t>scraped_markdown/automotiveworld/commercial-vehicle.md</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2637,7 +2625,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Section landing page is dominated by listing content rather than a full article.</t>
+          <t>Topic page is dominated by listing content and lacks substantive article narrative.</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -2650,17 +2638,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/e-mobility/</t>
+          <t>https://www.automotiveworld.com/data/</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-04-01T16:29:45+00:00</t>
+          <t>2026-03-31T15:32:04+00:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/e-mobility.md</t>
+          <t>scraped_markdown/automotiveworld/data.md</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2678,7 +2666,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Topic page is dominated by listing content and lacks substantive article narrative.</t>
+          <t>Section landing page is dominated by listing content rather than a full article.</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -2691,17 +2679,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/manufacturing/</t>
+          <t>https://www.automotiveworld.com/topics/e-mobility/</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-04-01T14:09:18+00:00</t>
+          <t>2026-04-01T16:29:45+00:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/manufacturing.md</t>
+          <t>scraped_markdown/automotiveworld/e-mobility.md</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2732,17 +2720,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/markets/</t>
+          <t>https://www.automotiveworld.com/topics/manufacturing/</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-04-01T15:03:02+00:00</t>
+          <t>2026-04-01T14:09:18+00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/markets.md</t>
+          <t>scraped_markdown/automotiveworld/manufacturing.md</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2773,17 +2761,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/news/</t>
+          <t>https://www.automotiveworld.com/topics/markets/</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-04-01T16:29:45+00:00</t>
+          <t>2026-04-01T15:03:02+00:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/news.md</t>
+          <t>scraped_markdown/automotiveworld/markets.md</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2801,7 +2789,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Section landing page is dominated by listing content rather than a full article.</t>
+          <t>Topic page is dominated by listing content and lacks substantive article narrative.</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
@@ -2814,7 +2802,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/oems/</t>
+          <t>https://www.automotiveworld.com/news/</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2824,7 +2812,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/oems.md</t>
+          <t>scraped_markdown/automotiveworld/news.md</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2842,7 +2830,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Topic page is dominated by listing content and lacks substantive article narrative.</t>
+          <t>Section landing page is dominated by listing content rather than a full article.</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
@@ -2855,17 +2843,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/data/sales/</t>
+          <t>https://www.automotiveworld.com/topics/oems/</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-03-31T15:32:04+00:00</t>
+          <t>2026-04-01T16:29:45+00:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/sales.md</t>
+          <t>scraped_markdown/automotiveworld/oems.md</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2883,7 +2871,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Page is dominated by dates, schedule blocks, or promotional/listing content.</t>
+          <t>Topic page is dominated by listing content and lacks substantive article narrative.</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -2896,17 +2884,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/topics/software-defined-vehicle/</t>
+          <t>https://www.automotiveworld.com/partner-content/</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-04-01T15:03:02+00:00</t>
+          <t>2026-04-02T06:34:35+00:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/software-defined-vehicle.md</t>
+          <t>scraped_markdown/automotiveworld/partner-content.md</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2924,7 +2912,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Topic page is dominated by listing content and lacks substantive article narrative.</t>
+          <t>Section landing page is dominated by listing content rather than a full article.</t>
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
@@ -2937,17 +2925,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.automotiveworld.com/file-tag/data/</t>
+          <t>https://www.automotiveworld.com/data/sales/</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-03-31T09:35:12+00:00</t>
+          <t>2026-03-31T15:32:04+00:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>scraped_markdown/automotiveworld/data_61.md</t>
+          <t>scraped_markdown/automotiveworld/sales.md</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2956,7 +2944,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -2965,11 +2953,93 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Body is just a date-based archive list with no article narrative or engineering content.</t>
+          <t>Page is dominated by dates, schedule blocks, or promotional/listing content.</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
+        <is>
+          <t>skipped_not_selected</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>https://www.automotiveworld.com/topics/software-defined-vehicle/</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-04-02T06:34:35+00:00</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>scraped_markdown/automotiveworld/software-defined-vehicle.md</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>10</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Topic page is dominated by listing content and lacks substantive article narrative.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>skipped_not_selected</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>https://www.automotiveworld.com/file-tag/data/</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-03-31T09:35:12+00:00</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>scraped_markdown/automotiveworld/data_63.md</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>not_selected</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Body is just a date archive with no article narrative or engineering content.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
         <is>
           <t>skipped_not_selected</t>
         </is>

</xml_diff>